<commit_message>
Updated gear and metier codes
</commit_message>
<xml_diff>
--- a/Metiers/Reference_lists/Code-ERSGearType-v1.1.xlsx
+++ b/Metiers/Reference_lists/Code-ERSGearType-v1.1.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\joeg\Github\RCGs\Metiers\Reference_lists\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sébastien\Dossiers_courant\_WK_METIER_20180122\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8BEF91-A44D-403D-A134-1933D4A5AB7D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13440" windowHeight="6990" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="formatted" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">formatted!$A$1:$F$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">formatted!$A$1:$F$69</definedName>
     <definedName name="OLE_LINK7" localSheetId="1">formatted!#REF!</definedName>
     <definedName name="OLE_LINK7" localSheetId="0">Sheet1!$B$6</definedName>
   </definedNames>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="190">
   <si>
     <t>Code</t>
   </si>
@@ -583,12 +584,24 @@
   </si>
   <si>
     <t>LDF,NSEA,Natl</t>
+  </si>
+  <si>
+    <t>OTS</t>
+  </si>
+  <si>
+    <t>Twin otter trawls for shrimps</t>
+  </si>
+  <si>
+    <t>HMP</t>
+  </si>
+  <si>
+    <t>Harvesting pumps</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -639,7 +652,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -694,8 +707,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1039,11 +1058,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1054,14 +1165,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1088,9 +1195,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1115,9 +1219,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1160,9 +1261,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1199,9 +1297,6 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -1227,9 +1322,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1239,16 +1331,16 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1281,10 +1373,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1302,7 +1394,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1347,9 +1439,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -1395,37 +1484,34 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1440,6 +1526,89 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1458,9 +1627,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Kontor">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1498,7 +1667,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Kontor">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1533,6 +1702,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1568,9 +1754,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Kontor">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1743,469 +1946,428 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F53"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="33.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="33.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="42.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="36.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6328125" customWidth="1"/>
+    <col min="2" max="2" width="42.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36.453125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C2" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>84</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="6"/>
-    </row>
-    <row r="6" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="14" t="s">
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="C6" s="5"/>
+    </row>
+    <row r="7" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="C7" s="5"/>
+    </row>
+    <row r="8" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="C8" s="5"/>
+    </row>
+    <row r="9" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="C9" s="5"/>
+    </row>
+    <row r="10" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="14" t="s">
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9"/>
+      <c r="B11" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="C11" s="5"/>
+    </row>
+    <row r="12" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="C12" s="5"/>
+    </row>
+    <row r="13" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="7"/>
-    </row>
-    <row r="14" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="C13" s="5"/>
+    </row>
+    <row r="14" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="7"/>
-    </row>
-    <row r="15" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="C14" s="5"/>
+    </row>
+    <row r="15" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="C15" s="5"/>
+    </row>
+    <row r="16" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14" t="s">
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="11"/>
+      <c r="B17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="7"/>
-    </row>
-    <row r="18" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10" t="s">
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9"/>
+      <c r="B18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="7"/>
-    </row>
-    <row r="19" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="7"/>
-    </row>
-    <row r="20" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="7"/>
-    </row>
-    <row r="21" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="7"/>
-    </row>
-    <row r="22" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="C21" s="5"/>
+    </row>
+    <row r="22" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="7"/>
-    </row>
-    <row r="23" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="C22" s="5"/>
+    </row>
+    <row r="23" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
+      <c r="C23" s="5"/>
+    </row>
+    <row r="24" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="7"/>
-    </row>
-    <row r="25" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10" t="s">
+      <c r="C24" s="5"/>
+    </row>
+    <row r="25" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="7"/>
-    </row>
-    <row r="26" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+      <c r="C25" s="5"/>
+    </row>
+    <row r="26" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="7"/>
-    </row>
-    <row r="27" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="C26" s="5"/>
+    </row>
+    <row r="27" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="7"/>
-    </row>
-    <row r="28" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
+      <c r="C27" s="5"/>
+    </row>
+    <row r="28" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="7"/>
-    </row>
-    <row r="29" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="14" t="s">
+      <c r="C28" s="5"/>
+    </row>
+    <row r="29" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="11" t="s">
+    </row>
+    <row r="30" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="5"/>
-      <c r="D30" s="4"/>
-    </row>
-    <row r="31" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="12"/>
-      <c r="B31" s="14" t="s">
+    </row>
+    <row r="31" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
+      <c r="B31" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="11" t="s">
+    </row>
+    <row r="32" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="5"/>
-      <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="11" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="5"/>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="11" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="4"/>
-    </row>
-    <row r="36" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="11" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="11" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="4"/>
-    </row>
-    <row r="38" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="12"/>
-      <c r="B38" s="14" t="s">
+    </row>
+    <row r="38" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10"/>
+      <c r="B38" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="5"/>
-      <c r="D38" s="4"/>
-    </row>
-    <row r="39" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="11" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="40" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="11" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="4"/>
-    </row>
-    <row r="41" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="12"/>
-      <c r="B41" s="14" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="4"/>
-    </row>
-    <row r="42" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="11" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="4"/>
-    </row>
-    <row r="43" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="11" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C43" s="5"/>
-      <c r="D43" s="4"/>
-    </row>
-    <row r="44" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="11" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="4"/>
-    </row>
-    <row r="45" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="11" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="4"/>
-    </row>
-    <row r="46" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="11" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C46" s="5"/>
-      <c r="D46" s="4"/>
-    </row>
-    <row r="47" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="11" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C47" s="5"/>
-      <c r="D47" s="4"/>
-    </row>
-    <row r="48" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="11" t="s">
+    </row>
+    <row r="48" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="4"/>
-    </row>
-    <row r="49" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="12"/>
-      <c r="B49" s="14" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="10"/>
+      <c r="B49" s="12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="11" t="s">
+    <row r="50" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="13" t="s">
+    <row r="51" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B51" s="10" t="s">
+      <c r="B51" s="8" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="13" t="s">
+    <row r="52" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B52" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="13" t="s">
+    <row r="53" spans="1:2" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="8" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2218,1448 +2380,1490 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J67"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="33.75" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J69"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="33.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.140625" customWidth="1"/>
-    <col min="2" max="2" width="63.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.140625" style="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.7109375" style="17"/>
-    <col min="10" max="10" width="39.42578125" style="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" customWidth="1"/>
+    <col min="2" max="2" width="63.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.54296875" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.54296875" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.08984375" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" style="14"/>
+    <col min="10" max="10" width="39.453125" style="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:10" ht="15.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="39" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="F1" s="123" t="s">
+      <c r="F1" s="114" t="s">
         <v>180</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="39" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="71" t="s">
+    <row r="2" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="64" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="65" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="73" t="s">
+      <c r="C2" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="74" t="s">
+      <c r="D2" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="75" t="s">
+      <c r="E2" s="68" t="s">
         <v>178</v>
       </c>
-      <c r="F2" s="124" t="s">
+      <c r="F2" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G2" s="68"/>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="32" t="s">
+      <c r="G2" s="61"/>
+    </row>
+    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A3" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="55" t="s">
+      <c r="D3" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="64"/>
-      <c r="F3" s="125" t="s">
+      <c r="E3" s="57"/>
+      <c r="F3" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G3" s="67"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="21" t="s">
+      <c r="G3" s="60"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="18" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="76" t="s">
+    <row r="4" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="69" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="77" t="s">
+      <c r="B4" s="70" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="78" t="s">
+      <c r="C4" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="79" t="s">
+      <c r="D4" s="72" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="80"/>
-      <c r="F4" s="126" t="s">
+      <c r="E4" s="73"/>
+      <c r="F4" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G4" s="81"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="21" t="s">
+      <c r="G4" s="74"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="18" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="83" t="s">
+    <row r="5" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="77" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="85" t="s">
+      <c r="C5" s="78" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="86" t="s">
+      <c r="D5" s="79" t="s">
         <v>76</v>
       </c>
-      <c r="E5" s="87" t="s">
+      <c r="E5" s="80" t="s">
         <v>178</v>
       </c>
-      <c r="F5" s="127" t="s">
+      <c r="F5" s="118" t="s">
         <v>182</v>
       </c>
-      <c r="G5" s="88" t="s">
+      <c r="G5" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="21" t="s">
+      <c r="I5" s="20"/>
+      <c r="J5" s="18" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="71" t="s">
+    <row r="6" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="64" t="s">
         <v>132</v>
       </c>
-      <c r="B6" s="72" t="s">
+      <c r="B6" s="65" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="73" t="s">
+      <c r="C6" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="89" t="s">
+      <c r="D6" s="82" t="s">
         <v>132</v>
       </c>
-      <c r="E6" s="89" t="s">
+      <c r="E6" s="82" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="128" t="s">
+      <c r="F6" s="119" t="s">
         <v>182</v>
       </c>
-      <c r="G6" s="88" t="s">
+      <c r="G6" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25" t="s">
+      <c r="I6" s="21"/>
+      <c r="J6" s="18" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="56" t="s">
+      <c r="D7" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="E7" s="58" t="s">
+      <c r="E7" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="F7" s="129" t="s">
+      <c r="F7" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G7" s="88" t="s">
+      <c r="G7" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="25" t="s">
+      <c r="I7" s="22"/>
+      <c r="J7" s="18" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+    <row r="8" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="58" t="s">
+      <c r="E8" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="F8" s="129" t="s">
+      <c r="F8" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G8" s="88" t="s">
+      <c r="G8" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+    <row r="9" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A9" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="132" t="s">
+      <c r="D9" s="123" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="133"/>
-      <c r="F9" s="125" t="s">
+      <c r="E9" s="124"/>
+      <c r="F9" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="67"/>
-    </row>
-    <row r="10" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
+      <c r="G9" s="60"/>
+    </row>
+    <row r="10" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="55" t="s">
+      <c r="D10" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="64"/>
-      <c r="F10" s="125" t="s">
+      <c r="E10" s="57"/>
+      <c r="F10" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G10" s="67"/>
-    </row>
-    <row r="11" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+      <c r="G10" s="60"/>
+    </row>
+    <row r="11" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="55" t="s">
+      <c r="D11" s="49" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="64"/>
-      <c r="F11" s="125" t="s">
+      <c r="E11" s="57"/>
+      <c r="F11" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G11" s="88" t="s">
+      <c r="G11" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32" t="s">
+    <row r="12" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="56" t="s">
+      <c r="D12" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="58" t="s">
+      <c r="E12" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="F12" s="129" t="s">
+      <c r="F12" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G12" s="88" t="s">
+      <c r="G12" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="90" t="s">
+    <row r="13" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="91" t="s">
+      <c r="B13" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="92" t="s">
+      <c r="C13" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="93" t="s">
+      <c r="D13" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="E13" s="94"/>
-      <c r="F13" s="126" t="s">
+      <c r="E13" s="87"/>
+      <c r="F13" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G13" s="81"/>
-    </row>
-    <row r="14" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="95" t="s">
+      <c r="G13" s="74"/>
+    </row>
+    <row r="14" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="88" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="96" t="s">
+      <c r="B14" s="89" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="97" t="s">
+      <c r="C14" s="90" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="98" t="s">
+      <c r="D14" s="91" t="s">
         <v>110</v>
       </c>
-      <c r="E14" s="99"/>
-      <c r="F14" s="127" t="s">
+      <c r="E14" s="92"/>
+      <c r="F14" s="118" t="s">
         <v>181</v>
       </c>
-      <c r="G14" s="88"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="100" t="s">
+      <c r="G14" s="81"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A15" s="93" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="101" t="s">
+      <c r="B15" s="94" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="102" t="s">
+      <c r="C15" s="95" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="103" t="s">
+      <c r="D15" s="96" t="s">
         <v>75</v>
       </c>
-      <c r="E15" s="104"/>
-      <c r="F15" s="124" t="s">
+      <c r="E15" s="97"/>
+      <c r="F15" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G15" s="68"/>
-    </row>
-    <row r="16" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="76" t="s">
+      <c r="G15" s="61"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A16" s="139" t="s">
         <v>113</v>
       </c>
-      <c r="B16" s="77" t="s">
+      <c r="B16" s="140" t="s">
         <v>114</v>
       </c>
-      <c r="C16" s="78" t="s">
+      <c r="C16" s="141" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="105" t="s">
+      <c r="D16" s="142" t="s">
         <v>113</v>
       </c>
-      <c r="E16" s="94"/>
-      <c r="F16" s="126" t="s">
+      <c r="E16" s="143"/>
+      <c r="F16" s="144" t="s">
         <v>181</v>
       </c>
-      <c r="G16" s="81"/>
-    </row>
-    <row r="17" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="71" t="s">
+      <c r="G16" s="145"/>
+    </row>
+    <row r="17" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="146" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="147" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="148" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="149" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" s="150"/>
+      <c r="F17" s="151" t="s">
+        <v>181</v>
+      </c>
+      <c r="G17" s="152"/>
+    </row>
+    <row r="18" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="72" t="s">
+      <c r="B18" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C18" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="106" t="s">
+      <c r="D18" s="98" t="s">
         <v>115</v>
       </c>
-      <c r="E17" s="104"/>
-      <c r="F17" s="124" t="s">
+      <c r="E18" s="97"/>
+      <c r="F18" s="115" t="s">
         <v>182</v>
       </c>
-      <c r="G17" s="88" t="s">
+      <c r="G18" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32" t="s">
+    <row r="19" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="33" t="s">
+      <c r="B19" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="46" t="s">
+      <c r="C19" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="55" t="s">
+      <c r="D19" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="64"/>
-      <c r="F18" s="125" t="s">
+      <c r="E19" s="57"/>
+      <c r="F19" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G18" s="88" t="s">
+      <c r="G19" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32" t="s">
+    <row r="20" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B20" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="C19" s="46" t="s">
+      <c r="C20" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="55" t="s">
+      <c r="D20" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="E19" s="64"/>
-      <c r="F19" s="125" t="s">
+      <c r="E20" s="57"/>
+      <c r="F20" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G19" s="88" t="s">
+      <c r="G20" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32" t="s">
+    <row r="21" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="33" t="s">
+      <c r="B21" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="46" t="s">
+      <c r="C21" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="56" t="s">
+      <c r="D21" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="58" t="s">
+      <c r="E21" s="52" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="129" t="s">
+      <c r="F21" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G20" s="88" t="s">
+      <c r="G21" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+    <row r="22" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B22" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="46" t="s">
+      <c r="C22" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="55" t="s">
+      <c r="D22" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="64"/>
-      <c r="F21" s="125" t="s">
+      <c r="E22" s="57"/>
+      <c r="F22" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G21" s="88" t="s">
+      <c r="G22" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="30" t="s">
+    <row r="23" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B23" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="45" t="s">
+      <c r="C23" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="54" t="s">
+      <c r="D23" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="65" t="s">
+      <c r="E23" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F22" s="125" t="s">
+      <c r="F23" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G22" s="88" t="s">
+      <c r="G23" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
+    <row r="24" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B24" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="46" t="s">
+      <c r="C24" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="55" t="s">
+      <c r="D24" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="E23" s="64"/>
-      <c r="F23" s="125" t="s">
+      <c r="E24" s="57"/>
+      <c r="F24" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G23" s="88" t="s">
+      <c r="G24" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32" t="s">
+    <row r="25" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="33" t="s">
+      <c r="B25" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="46" t="s">
+      <c r="C25" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="55" t="s">
+      <c r="D25" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="64"/>
-      <c r="F24" s="125" t="s">
+      <c r="E25" s="57"/>
+      <c r="F25" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G24" s="67"/>
-    </row>
-    <row r="25" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
+      <c r="G25" s="60"/>
+    </row>
+    <row r="26" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B26" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="C25" s="45" t="s">
+      <c r="C26" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D25" s="54" t="s">
+      <c r="D26" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="65" t="s">
+      <c r="E26" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F25" s="125" t="s">
+      <c r="F26" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G25" s="88" t="s">
+      <c r="G26" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="34" t="s">
+    <row r="27" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="35" t="s">
+      <c r="B27" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="C26" s="47" t="s">
+      <c r="C27" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="57" t="s">
+      <c r="D27" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="E26" s="65" t="s">
+      <c r="E27" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F26" s="125" t="s">
+      <c r="F27" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G26" s="88" t="s">
+      <c r="G27" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="107" t="s">
+    <row r="28" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="108" t="s">
+      <c r="B28" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="C27" s="109" t="s">
+      <c r="C28" s="101" t="s">
         <v>34</v>
       </c>
-      <c r="D27" s="66" t="s">
+      <c r="D28" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="E27" s="66" t="s">
+      <c r="E28" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="130" t="s">
+      <c r="F28" s="121" t="s">
         <v>182</v>
       </c>
-      <c r="G27" s="88" t="s">
+      <c r="G28" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A28" s="71" t="s">
+    <row r="29" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A29" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="B28" s="72" t="s">
+      <c r="B29" s="65" t="s">
         <v>121</v>
       </c>
-      <c r="C28" s="73" t="s">
+      <c r="C29" s="66" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="106" t="s">
+      <c r="D29" s="98" t="s">
         <v>117</v>
       </c>
-      <c r="E28" s="104"/>
-      <c r="F28" s="124" t="s">
+      <c r="E29" s="97"/>
+      <c r="F29" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G28" s="68"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="34" t="s">
+      <c r="G29" s="61"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A30" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="B29" s="35" t="s">
+      <c r="B30" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="47" t="s">
+      <c r="C30" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="D29" s="57" t="s">
+      <c r="D30" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="E29" s="65" t="s">
+      <c r="E30" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F29" s="125" t="s">
+      <c r="F30" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G29" s="67"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="34" t="s">
+      <c r="G30" s="60"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A31" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="35" t="s">
+      <c r="B31" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="C30" s="47" t="s">
+      <c r="C31" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="57" t="s">
+      <c r="D31" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="E30" s="65" t="s">
+      <c r="E31" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F30" s="125" t="s">
+      <c r="F31" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G30" s="67"/>
-    </row>
-    <row r="31" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="42" t="s">
+      <c r="G31" s="60"/>
+    </row>
+    <row r="32" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="B31" s="43" t="s">
+      <c r="B32" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="110" t="s">
+      <c r="C32" s="102" t="s">
         <v>118</v>
       </c>
-      <c r="D31" s="111" t="s">
+      <c r="D32" s="103" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="80" t="s">
+      <c r="E32" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="F31" s="126" t="s">
+      <c r="F32" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G31" s="81"/>
-    </row>
-    <row r="32" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="112" t="s">
+      <c r="G32" s="74"/>
+    </row>
+    <row r="33" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="104" t="s">
         <v>76</v>
       </c>
-      <c r="B32" s="113" t="s">
+      <c r="B33" s="105" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="85" t="s">
+      <c r="C33" s="78" t="s">
         <v>80</v>
       </c>
-      <c r="D32" s="114" t="s">
+      <c r="D33" s="106" t="s">
         <v>76</v>
       </c>
-      <c r="E32" s="99"/>
-      <c r="F32" s="127" t="s">
+      <c r="E33" s="92"/>
+      <c r="F33" s="118" t="s">
         <v>182</v>
       </c>
-      <c r="G32" s="88" t="s">
+      <c r="G33" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="112" t="s">
+    <row r="34" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="104" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="113" t="s">
+      <c r="B34" s="105" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="115" t="s">
+      <c r="C34" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="D33" s="116" t="s">
+      <c r="D34" s="108" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="137"/>
-      <c r="F33" s="127" t="s">
+      <c r="E34" s="128"/>
+      <c r="F34" s="118" t="s">
         <v>182</v>
       </c>
-      <c r="G33" s="88" t="s">
+      <c r="G34" s="81" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="71" t="s">
+    <row r="35" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A35" s="64" t="s">
         <v>94</v>
       </c>
-      <c r="B34" s="72" t="s">
+      <c r="B35" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="73" t="s">
+      <c r="C35" s="66" t="s">
         <v>101</v>
       </c>
-      <c r="D34" s="106" t="s">
+      <c r="D35" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="E34" s="104"/>
-      <c r="F34" s="124" t="s">
+      <c r="E35" s="97"/>
+      <c r="F35" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="68"/>
-    </row>
-    <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="34" t="s">
+      <c r="G35" s="61"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A36" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="35" t="s">
+      <c r="B36" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="C35" s="47" t="s">
+      <c r="C36" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="D35" s="57" t="s">
+      <c r="D36" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="E35" s="65" t="s">
+      <c r="E36" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F35" s="125" t="s">
+      <c r="F36" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G35" s="67"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A36" s="34" t="s">
+      <c r="G36" s="60"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A37" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="B36" s="35" t="s">
+      <c r="B37" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="C36" s="47" t="s">
+      <c r="C37" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="D36" s="59" t="s">
+      <c r="D37" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="E36" s="64"/>
-      <c r="F36" s="125" t="s">
+      <c r="E37" s="57"/>
+      <c r="F37" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G36" s="67"/>
-    </row>
-    <row r="37" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="42" t="s">
+      <c r="G37" s="60"/>
+    </row>
+    <row r="38" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="B37" s="43" t="s">
+      <c r="B38" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="C37" s="110" t="s">
+      <c r="C38" s="102" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="111" t="s">
+      <c r="D38" s="103" t="s">
         <v>94</v>
       </c>
-      <c r="E37" s="80" t="s">
+      <c r="E38" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="F37" s="126" t="s">
+      <c r="F38" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G37" s="81"/>
-    </row>
-    <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A38" s="71" t="s">
+      <c r="G38" s="74"/>
+    </row>
+    <row r="39" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A39" s="64" t="s">
         <v>126</v>
       </c>
-      <c r="B38" s="72" t="s">
+      <c r="B39" s="65" t="s">
         <v>127</v>
       </c>
-      <c r="C38" s="73" t="s">
+      <c r="C39" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="D38" s="106" t="s">
+      <c r="D39" s="98" t="s">
         <v>126</v>
       </c>
-      <c r="E38" s="104"/>
-      <c r="F38" s="124" t="s">
+      <c r="E39" s="97"/>
+      <c r="F39" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G38" s="68"/>
-    </row>
-    <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A39" s="36" t="s">
+      <c r="G39" s="61"/>
+    </row>
+    <row r="40" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A40" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="B39" s="37" t="s">
+      <c r="B40" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="C39" s="48" t="s">
+      <c r="C40" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D39" s="60" t="s">
+      <c r="D40" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="E39" s="64"/>
-      <c r="F39" s="125" t="s">
+      <c r="E40" s="57"/>
+      <c r="F40" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G39" s="67"/>
-    </row>
-    <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A40" s="36" t="s">
+      <c r="G40" s="60"/>
+    </row>
+    <row r="41" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A41" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="B41" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="C40" s="48" t="s">
+      <c r="C41" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D40" s="134" t="s">
+      <c r="D41" s="125" t="s">
         <v>50</v>
       </c>
-      <c r="E40" s="133"/>
-      <c r="F40" s="125" t="s">
+      <c r="E41" s="124"/>
+      <c r="F41" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G40" s="67"/>
-    </row>
-    <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A41" s="36" t="s">
+      <c r="G41" s="60"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A42" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="B41" s="37" t="s">
+      <c r="B42" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="C41" s="48" t="s">
+      <c r="C42" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D41" s="60" t="s">
+      <c r="D42" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="E41" s="64"/>
-      <c r="F41" s="125" t="s">
+      <c r="E42" s="57"/>
+      <c r="F42" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G41" s="67"/>
-    </row>
-    <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="36" t="s">
+      <c r="G42" s="60"/>
+    </row>
+    <row r="43" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A43" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="37" t="s">
+      <c r="B43" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="C42" s="48" t="s">
+      <c r="C43" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="60" t="s">
+      <c r="D43" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="64"/>
-      <c r="F42" s="125" t="s">
+      <c r="E43" s="57"/>
+      <c r="F43" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G42" s="67"/>
-    </row>
-    <row r="43" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="107" t="s">
+      <c r="G43" s="60"/>
+    </row>
+    <row r="44" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="99" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="108" t="s">
+      <c r="B44" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="C43" s="109" t="s">
+      <c r="C44" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="D43" s="66" t="s">
+      <c r="D44" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="E43" s="66" t="s">
+      <c r="E44" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="F43" s="130" t="s">
+      <c r="F44" s="121" t="s">
         <v>181</v>
       </c>
-      <c r="G43" s="70"/>
-    </row>
-    <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A44" s="100" t="s">
+      <c r="G44" s="63"/>
+    </row>
+    <row r="45" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A45" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="B44" s="101" t="s">
+      <c r="B45" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="102" t="s">
+      <c r="C45" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="D44" s="135" t="s">
+      <c r="D45" s="126" t="s">
         <v>46</v>
       </c>
-      <c r="E44" s="136"/>
-      <c r="F44" s="124" t="s">
+      <c r="E45" s="127"/>
+      <c r="F45" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G44" s="68"/>
-    </row>
-    <row r="45" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A45" s="36" t="s">
+      <c r="G45" s="61"/>
+    </row>
+    <row r="46" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A46" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="37" t="s">
+      <c r="B46" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="C45" s="48" t="s">
+      <c r="C46" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="D45" s="60" t="s">
+      <c r="D46" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="E45" s="64"/>
-      <c r="F45" s="125" t="s">
+      <c r="E46" s="57"/>
+      <c r="F46" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G45" s="67"/>
-    </row>
-    <row r="46" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A46" s="36" t="s">
+      <c r="G46" s="60"/>
+    </row>
+    <row r="47" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A47" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="37" t="s">
+      <c r="B47" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="C46" s="48" t="s">
+      <c r="C47" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="D46" s="61" t="s">
+      <c r="D47" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="E46" s="65" t="s">
+      <c r="E47" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F46" s="125" t="s">
+      <c r="F47" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G46" s="67"/>
-    </row>
-    <row r="47" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="107" t="s">
+      <c r="G47" s="60"/>
+    </row>
+    <row r="48" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="99" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="108" t="s">
+      <c r="B48" s="100" t="s">
         <v>145</v>
       </c>
-      <c r="C47" s="109" t="s">
+      <c r="C48" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="D47" s="117" t="s">
+      <c r="D48" s="109" t="s">
         <v>43</v>
       </c>
-      <c r="E47" s="80" t="s">
+      <c r="E48" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="F47" s="126" t="s">
+      <c r="F48" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G47" s="81"/>
-    </row>
-    <row r="48" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A48" s="100" t="s">
+      <c r="G48" s="74"/>
+    </row>
+    <row r="49" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A49" s="93" t="s">
         <v>68</v>
       </c>
-      <c r="B48" s="101" t="s">
+      <c r="B49" s="94" t="s">
         <v>33</v>
       </c>
-      <c r="C48" s="102" t="s">
+      <c r="C49" s="95" t="s">
         <v>31</v>
       </c>
-      <c r="D48" s="120" t="s">
+      <c r="D49" s="112" t="s">
         <v>107</v>
       </c>
-      <c r="E48" s="121" t="s">
+      <c r="E49" s="68" t="s">
         <v>178</v>
       </c>
-      <c r="F48" s="124" t="s">
+      <c r="F49" s="115" t="s">
         <v>181</v>
       </c>
-      <c r="G48" s="68"/>
-    </row>
-    <row r="49" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A49" s="38" t="s">
+      <c r="G49" s="61"/>
+    </row>
+    <row r="50" spans="1:10" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="B49" s="39" t="s">
+      <c r="B50" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="C49" s="49" t="s">
+      <c r="C50" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="D49" s="58" t="s">
+      <c r="D50" s="52" t="s">
         <v>171</v>
       </c>
-      <c r="E49" s="58" t="s">
+      <c r="E50" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="F49" s="129" t="s">
+      <c r="F50" s="120" t="s">
         <v>181</v>
       </c>
-      <c r="G49" s="69"/>
-    </row>
-    <row r="50" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A50" s="34" t="s">
+      <c r="G50" s="62"/>
+    </row>
+    <row r="51" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A51" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="B50" s="35" t="s">
+      <c r="B51" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="C50" s="47" t="s">
+      <c r="C51" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="D50" s="59" t="s">
+      <c r="D51" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="E50" s="64"/>
-      <c r="F50" s="125" t="s">
+      <c r="E51" s="57"/>
+      <c r="F51" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G50" s="67"/>
-    </row>
-    <row r="51" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A51" s="36" t="s">
+      <c r="G51" s="60"/>
+    </row>
+    <row r="52" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A52" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="B51" s="37" t="s">
+      <c r="B52" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="C51" s="48" t="s">
+      <c r="C52" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="D51" s="60" t="s">
+      <c r="D52" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="E51" s="64"/>
-      <c r="F51" s="125" t="s">
+      <c r="E52" s="57"/>
+      <c r="F52" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G51" s="67"/>
-    </row>
-    <row r="52" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A52" s="34" t="s">
+      <c r="G52" s="60"/>
+    </row>
+    <row r="53" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A53" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="35" t="s">
+      <c r="B53" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="47" t="s">
+      <c r="C53" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="D52" s="59" t="s">
+      <c r="D53" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="E52" s="64"/>
-      <c r="F52" s="125" t="s">
+      <c r="E53" s="57"/>
+      <c r="F53" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G52" s="67"/>
-    </row>
-    <row r="53" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="42" t="s">
+      <c r="G53" s="60"/>
+    </row>
+    <row r="54" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="B53" s="43" t="s">
+      <c r="B54" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="C53" s="110" t="s">
+      <c r="C54" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="D53" s="122" t="s">
+      <c r="D54" s="113" t="s">
         <v>107</v>
       </c>
-      <c r="E53" s="94"/>
-      <c r="F53" s="126" t="s">
+      <c r="E54" s="87"/>
+      <c r="F54" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="G53" s="81"/>
-    </row>
-    <row r="54" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A54" s="30" t="s">
+      <c r="G54" s="74"/>
+    </row>
+    <row r="55" spans="1:10" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="31" t="s">
+      <c r="B55" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="C54" s="118" t="s">
+      <c r="C55" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="D54" s="119" t="s">
+      <c r="D55" s="111" t="s">
         <v>140</v>
       </c>
-      <c r="E54" s="56" t="s">
+      <c r="E55" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="F54" s="131" t="s">
+      <c r="F55" s="122" t="s">
         <v>182</v>
       </c>
-      <c r="G54" s="82" t="s">
+      <c r="G55" s="75" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A55" s="36" t="s">
+    <row r="56" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A56" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="40" t="s">
+      <c r="B56" s="36" t="s">
         <v>151</v>
       </c>
-      <c r="C55" s="51" t="s">
+      <c r="C56" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="60" t="s">
+      <c r="D56" s="54" t="s">
         <v>53</v>
       </c>
-      <c r="E55" s="64"/>
-      <c r="F55" s="125" t="s">
+      <c r="E56" s="57"/>
+      <c r="F56" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G55" s="67" t="s">
+      <c r="G56" s="60" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A56" s="36" t="s">
+    <row r="57" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A57" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="B56" s="41" t="s">
+      <c r="B57" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="C56" s="51" t="s">
+      <c r="C57" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D56" s="60" t="s">
+      <c r="D57" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="E56" s="64"/>
-      <c r="F56" s="125" t="s">
+      <c r="E57" s="57"/>
+      <c r="F57" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G56" s="67" t="s">
+      <c r="G57" s="60" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A57" s="36" t="s">
+    <row r="58" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A58" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="37" t="s">
+      <c r="B58" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="C57" s="51" t="s">
+      <c r="C58" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D57" s="60" t="s">
+      <c r="D58" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="E57" s="64"/>
-      <c r="F57" s="125" t="s">
+      <c r="E58" s="138"/>
+      <c r="F58" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G57" s="67" t="s">
+      <c r="G58" s="60" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A58" s="36" t="s">
+    <row r="59" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A59" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="B58" s="37" t="s">
+      <c r="B59" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="C58" s="51" t="s">
+      <c r="C59" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D58" s="60" t="s">
+      <c r="D59" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="E58" s="64"/>
-      <c r="F58" s="125" t="s">
+      <c r="E59" s="57"/>
+      <c r="F59" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G58" s="67"/>
-    </row>
-    <row r="59" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A59" s="36" t="s">
+      <c r="G59" s="60"/>
+    </row>
+    <row r="60" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A60" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="B59" s="37" t="s">
+      <c r="B60" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="C59" s="51" t="s">
+      <c r="C60" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D59" s="60" t="s">
+      <c r="D60" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="E59" s="64"/>
-      <c r="F59" s="125" t="s">
+      <c r="E60" s="57"/>
+      <c r="F60" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G59" s="67"/>
-    </row>
-    <row r="60" spans="1:10" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A60" s="36" t="s">
+      <c r="G60" s="60"/>
+    </row>
+    <row r="61" spans="1:10" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="B60" s="37" t="s">
+      <c r="B61" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="C60" s="51" t="s">
+      <c r="C61" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D60" s="58" t="s">
+      <c r="D61" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="E60" s="58" t="s">
+      <c r="E61" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="F60" s="129" t="s">
+      <c r="F61" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G60" s="69" t="s">
+      <c r="G61" s="62" t="s">
         <v>183</v>
       </c>
-      <c r="H60"/>
-      <c r="I60" s="18"/>
-      <c r="J60" s="18"/>
-    </row>
-    <row r="61" spans="1:10" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A61" s="36" t="s">
+      <c r="H61"/>
+      <c r="I61" s="15"/>
+      <c r="J61" s="15"/>
+    </row>
+    <row r="62" spans="1:10" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A62" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="B61" s="37" t="s">
+      <c r="B62" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="C61" s="51" t="s">
+      <c r="C62" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D61" s="60" t="s">
+      <c r="D62" s="54" t="s">
         <v>52</v>
       </c>
-      <c r="E61" s="64"/>
-      <c r="F61" s="125" t="s">
+      <c r="E62" s="57"/>
+      <c r="F62" s="116" t="s">
         <v>181</v>
       </c>
-      <c r="G61" s="67"/>
-      <c r="H61"/>
-      <c r="I61" s="18"/>
-      <c r="J61" s="18"/>
-    </row>
-    <row r="62" spans="1:10" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A62" s="36" t="s">
+      <c r="G62" s="60"/>
+      <c r="H62"/>
+      <c r="I62" s="15"/>
+      <c r="J62" s="15"/>
+    </row>
+    <row r="63" spans="1:10" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A63" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B62" s="37" t="s">
+      <c r="B63" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="C62" s="51" t="s">
+      <c r="C63" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D62" s="61" t="s">
+      <c r="D63" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="E62" s="65" t="s">
+      <c r="E63" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F62" s="125" t="s">
+      <c r="F63" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G62" s="67" t="s">
+      <c r="G63" s="60" t="s">
         <v>183</v>
       </c>
-      <c r="H62"/>
-      <c r="I62" s="18"/>
-      <c r="J62" s="18"/>
-    </row>
-    <row r="63" spans="1:10" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A63" s="36" t="s">
+      <c r="H63"/>
+      <c r="I63" s="15"/>
+      <c r="J63" s="15"/>
+    </row>
+    <row r="64" spans="1:10" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A64" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="B63" s="37" t="s">
+      <c r="B64" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="C63" s="51" t="s">
+      <c r="C64" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D63" s="61" t="s">
+      <c r="D64" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="E63" s="65" t="s">
+      <c r="E64" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F63" s="125" t="s">
+      <c r="F64" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G63" s="67" t="s">
+      <c r="G64" s="60" t="s">
         <v>183</v>
       </c>
-      <c r="H63"/>
-      <c r="I63" s="18"/>
-      <c r="J63" s="18"/>
-    </row>
-    <row r="64" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A64" s="34" t="s">
+      <c r="H64"/>
+      <c r="I64" s="15"/>
+      <c r="J64" s="15"/>
+    </row>
+    <row r="65" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A65" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="B64" s="35" t="s">
+      <c r="B65" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="C64" s="50" t="s">
+      <c r="C65" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="61" t="s">
+      <c r="D65" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="E64" s="65" t="s">
+      <c r="E65" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="F64" s="125" t="s">
+      <c r="F65" s="116" t="s">
         <v>182</v>
       </c>
-      <c r="G64" s="67" t="s">
+      <c r="G65" s="60" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A65" s="38" t="s">
+    <row r="66" spans="1:7" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="B65" s="39" t="s">
+      <c r="B66" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="C65" s="52" t="s">
+      <c r="C66" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="D65" s="58" t="s">
+      <c r="D66" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="E65" s="58" t="s">
+      <c r="E66" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="F65" s="129" t="s">
+      <c r="F66" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="G65" s="69" t="s">
+      <c r="G66" s="62" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A66" s="34" t="s">
+    <row r="67" spans="1:7" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B66" s="35" t="s">
+      <c r="B67" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="C66" s="50" t="s">
+      <c r="C67" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="D66" s="62" t="s">
+      <c r="D67" s="56" t="s">
         <v>163</v>
       </c>
-      <c r="E66" s="58" t="s">
+      <c r="E67" s="52" t="s">
         <v>165</v>
       </c>
-      <c r="F66" s="129" t="s">
+      <c r="F67" s="120" t="s">
         <v>181</v>
       </c>
-      <c r="G66" s="69"/>
-    </row>
-    <row r="67" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="42" t="s">
+      <c r="G67" s="62"/>
+    </row>
+    <row r="68" spans="1:7" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A68" s="129" t="s">
         <v>166</v>
       </c>
-      <c r="B67" s="43" t="s">
+      <c r="B68" s="130" t="s">
         <v>167</v>
       </c>
-      <c r="C67" s="53" t="s">
+      <c r="C68" s="131" t="s">
         <v>14</v>
       </c>
-      <c r="D67" s="63" t="s">
+      <c r="D68" s="132" t="s">
         <v>166</v>
       </c>
-      <c r="E67" s="66" t="s">
+      <c r="E68" s="133" t="s">
         <v>168</v>
       </c>
-      <c r="F67" s="130" t="s">
+      <c r="F68" s="134" t="s">
         <v>182</v>
       </c>
-      <c r="G67" s="70" t="s">
+      <c r="G68" s="135" t="s">
         <v>183</v>
       </c>
     </row>
+    <row r="69" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="153" t="s">
+        <v>186</v>
+      </c>
+      <c r="B69" s="154" t="s">
+        <v>187</v>
+      </c>
+      <c r="C69" s="155" t="s">
+        <v>14</v>
+      </c>
+      <c r="D69" s="136" t="s">
+        <v>87</v>
+      </c>
+      <c r="E69" s="137" t="s">
+        <v>178</v>
+      </c>
+      <c r="F69" s="156" t="s">
+        <v>182</v>
+      </c>
+      <c r="G69" s="157" t="s">
+        <v>183</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:G61">
-    <sortCondition ref="C2:C61"/>
-    <sortCondition ref="A2:A61"/>
+  <sortState ref="A2:G62">
+    <sortCondition ref="C2:C62"/>
+    <sortCondition ref="A2:A62"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>